<commit_message>
Resumo de atividade — 4 de setembro de 2026
</commit_message>
<xml_diff>
--- a/Resumo_atividade/Resumo-survey_os_20260904.xlsx
+++ b/Resumo_atividade/Resumo-survey_os_20260904.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="245">
   <si>
     <t>Número</t>
   </si>
@@ -52,27 +52,78 @@
     <t>Abertura</t>
   </si>
   <si>
+    <t>OS-2026-0079</t>
+  </si>
+  <si>
+    <t>Atribuída</t>
+  </si>
+  <si>
+    <t>Alta</t>
+  </si>
+  <si>
+    <t>EVANDRO EDUARDO PIVA BIMONTI</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>Ouro Fino</t>
+  </si>
+  <si>
+    <t>SANTA ISABEL</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/g2xpSsCB96f143Ya7</t>
+  </si>
+  <si>
+    <t>-22.283309, -46.351726</t>
+  </si>
+  <si>
+    <t>MG (3001, 3002 e 3003)</t>
+  </si>
+  <si>
+    <t>Eric wesley Tavares</t>
+  </si>
+  <si>
+    <t>OS-2026-0078</t>
+  </si>
+  <si>
+    <t>Aberta</t>
+  </si>
+  <si>
+    <t>Média</t>
+  </si>
+  <si>
+    <t>RAFAEL DA ROCHA FLORENCIO DE PAULA</t>
+  </si>
+  <si>
+    <t>PR</t>
+  </si>
+  <si>
+    <t>Londrina</t>
+  </si>
+  <si>
+    <t>Jardim Vista Bela</t>
+  </si>
+  <si>
+    <t>Rua Eugênia Gonçalves Moreno, 99</t>
+  </si>
+  <si>
+    <t>-23.269158, -51.201915</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>OS-2026-0077</t>
   </si>
   <si>
-    <t>Atribuída</t>
-  </si>
-  <si>
-    <t>Média</t>
-  </si>
-  <si>
     <t>Willian Henrique Freire de Carvalho</t>
   </si>
   <si>
-    <t>PR</t>
-  </si>
-  <si>
     <t>Ivaiporã</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Rua Campo Grande</t>
   </si>
   <si>
@@ -88,9 +139,6 @@
     <t>Antonio Carlos Galvão Jorge</t>
   </si>
   <si>
-    <t>MG</t>
-  </si>
-  <si>
     <t>Itapeva</t>
   </si>
   <si>
@@ -100,9 +148,6 @@
     <t>-22.769906, -46.222698</t>
   </si>
   <si>
-    <t>MG (3001, 3002 e 3003)</t>
-  </si>
-  <si>
     <t>David Bossert Barbosa</t>
   </si>
   <si>
@@ -124,9 +169,6 @@
     <t>Crítica</t>
   </si>
   <si>
-    <t>EVANDRO EDUARDO PIVA BIMONTI</t>
-  </si>
-  <si>
     <t>Jacutinga</t>
   </si>
   <si>
@@ -142,9 +184,6 @@
     <t>Encerrada</t>
   </si>
   <si>
-    <t>Alta</t>
-  </si>
-  <si>
     <t>Estrada Municipal Doutor Nairo de Souza Vargas</t>
   </si>
   <si>
@@ -271,12 +310,6 @@
     <t>Allan Henrique da Silva</t>
   </si>
   <si>
-    <t>Londrina</t>
-  </si>
-  <si>
-    <t>Jardim Vista Bela</t>
-  </si>
-  <si>
     <t>Rua Braz Lucas Teruel, 108</t>
   </si>
   <si>
@@ -307,9 +340,6 @@
     <t>OS-2026-0059</t>
   </si>
   <si>
-    <t>RAFAEL DA ROCHA FLORENCIO DE PAULA</t>
-  </si>
-  <si>
     <t>Cambé</t>
   </si>
   <si>
@@ -404,9 +434,6 @@
   </si>
   <si>
     <t>-22.251445, -46.619643</t>
-  </si>
-  <si>
-    <t>Eric wesley Tavares</t>
   </si>
   <si>
     <t>OS-2026-0053</t>
@@ -1114,7 +1141,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M46"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1203,329 +1230,329 @@
         <v>22</v>
       </c>
       <c r="K2" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="L2" s="1">
-        <v>46271.125</v>
+        <v>46269.125</v>
       </c>
       <c r="M2" s="1">
-        <v>46269.55893490741</v>
+        <v>46269.68827564815</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E3" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="H3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="I3" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="J3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="K3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="L3" s="1">
-        <v>46270.125</v>
+        <v>46271.125</v>
       </c>
       <c r="M3" s="1">
-        <v>46268.99017603009</v>
+        <v>46269.66255648148</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="H4" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="I4" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="J4" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="K4" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="L4" s="1">
-        <v>46270.125</v>
+        <v>46271.125</v>
       </c>
       <c r="M4" s="1">
-        <v>46268.79206815972</v>
+        <v>46269.55893490741</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F5" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G5" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I5" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J5" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="K5" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="L5" s="1">
         <v>46270.125</v>
       </c>
       <c r="M5" s="1">
-        <v>46268.72042950231</v>
+        <v>46268.99017603009</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" t="s">
         <v>37</v>
       </c>
-      <c r="E6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" t="s">
-        <v>38</v>
-      </c>
-      <c r="G6" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" t="s">
-        <v>44</v>
-      </c>
       <c r="I6" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J6" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="K6" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="L6" s="1">
         <v>46270.125</v>
       </c>
       <c r="M6" s="1">
-        <v>46268.71752466435</v>
+        <v>46268.79206815972</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F7" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="G7" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="H7" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="I7" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="J7" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="K7" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="L7" s="1">
         <v>46270.125</v>
       </c>
       <c r="M7" s="1">
-        <v>46268.71495100694</v>
+        <v>46268.72042950231</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="D8" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="E8" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F8" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="G8" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="H8" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="I8" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="J8" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="K8" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="L8" s="1">
         <v>46270.125</v>
       </c>
       <c r="M8" s="1">
-        <v>46268.713350949074</v>
+        <v>46268.71752466435</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C9" t="s">
         <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F9" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="G9" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="H9" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="I9" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="J9" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="K9" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="L9" s="1">
         <v>46270.125</v>
       </c>
       <c r="M9" s="1">
-        <v>46268.56635226852</v>
+        <v>46268.71495100694</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>56</v>
       </c>
       <c r="C10" t="s">
         <v>15</v>
       </c>
       <c r="D10" t="s">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="E10" t="s">
         <v>17</v>
       </c>
       <c r="F10" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G10" t="s">
+        <v>33</v>
+      </c>
+      <c r="H10" t="s">
         <v>57</v>
       </c>
-      <c r="H10" t="s">
-        <v>58</v>
-      </c>
       <c r="I10" t="s">
-        <v>19</v>
+        <v>63</v>
       </c>
       <c r="J10" t="s">
         <v>22</v>
@@ -1537,276 +1564,276 @@
         <v>46270.125</v>
       </c>
       <c r="M10" s="1">
-        <v>46268.548608067125</v>
+        <v>46268.713350949074</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C11" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D11" t="s">
-        <v>61</v>
+        <v>16</v>
       </c>
       <c r="E11" t="s">
         <v>17</v>
       </c>
       <c r="F11" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="G11" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="H11" t="s">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="I11" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="J11" t="s">
         <v>22</v>
       </c>
       <c r="K11" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="L11" s="1">
         <v>46270.125</v>
       </c>
       <c r="M11" s="1">
-        <v>46268.53757355324</v>
+        <v>46268.56635226852</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="D12" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E12" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F12" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="G12" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H12" t="s">
-        <v>19</v>
+        <v>71</v>
       </c>
       <c r="I12" t="s">
-        <v>67</v>
+        <v>33</v>
       </c>
       <c r="J12" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="K12" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="L12" s="1">
-        <v>46267.125</v>
+        <v>46270.125</v>
       </c>
       <c r="M12" s="1">
-        <v>46267.78416134259</v>
+        <v>46268.548608067125</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C13" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D13" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E13" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F13" t="s">
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="G13" t="s">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="H13" t="s">
-        <v>73</v>
+        <v>37</v>
       </c>
       <c r="I13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J13" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="K13" t="s">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="L13" s="1">
-        <v>46269.125</v>
+        <v>46270.125</v>
       </c>
       <c r="M13" s="1">
-        <v>46267.65241516204</v>
+        <v>46268.53757355324</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C14" t="s">
         <v>15</v>
       </c>
       <c r="D14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E14" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F14" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H14" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="I14" t="s">
         <v>80</v>
       </c>
       <c r="J14" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="K14" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="L14" s="1">
-        <v>46266.125</v>
+        <v>46267.125</v>
       </c>
       <c r="M14" s="1">
-        <v>46265.609358125</v>
+        <v>46267.78416134259</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" t="s">
+        <v>83</v>
+      </c>
+      <c r="E15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" t="s">
+        <v>84</v>
+      </c>
+      <c r="G15" t="s">
+        <v>85</v>
+      </c>
+      <c r="H15" t="s">
+        <v>86</v>
+      </c>
+      <c r="I15" t="s">
+        <v>87</v>
+      </c>
+      <c r="J15" t="s">
+        <v>39</v>
+      </c>
+      <c r="K15" t="s">
         <v>81</v>
       </c>
-      <c r="B15" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15" t="s">
-        <v>32</v>
-      </c>
-      <c r="D15" t="s">
-        <v>76</v>
-      </c>
-      <c r="E15" t="s">
-        <v>25</v>
-      </c>
-      <c r="F15" t="s">
-        <v>77</v>
-      </c>
-      <c r="G15" t="s">
-        <v>78</v>
-      </c>
-      <c r="H15" t="s">
-        <v>82</v>
-      </c>
-      <c r="I15" t="s">
-        <v>83</v>
-      </c>
-      <c r="J15" t="s">
-        <v>29</v>
-      </c>
-      <c r="K15" t="s">
-        <v>76</v>
-      </c>
       <c r="L15" s="1">
-        <v>46265.125</v>
+        <v>46269.125</v>
       </c>
       <c r="M15" s="1">
-        <v>46265.60724832176</v>
+        <v>46267.65241516204</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C16" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D16" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="E16" t="s">
         <v>17</v>
       </c>
       <c r="F16" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G16" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="H16" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I16" t="s">
+        <v>93</v>
+      </c>
+      <c r="J16" t="s">
+        <v>22</v>
+      </c>
+      <c r="K16" t="s">
         <v>89</v>
-      </c>
-      <c r="J16" t="s">
-        <v>19</v>
-      </c>
-      <c r="K16" t="s">
-        <v>90</v>
       </c>
       <c r="L16" s="1">
         <v>46266.125</v>
       </c>
       <c r="M16" s="1">
-        <v>46264.545438518515</v>
+        <v>46265.609358125</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B17" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C17" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="D17" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="E17" t="s">
         <v>17</v>
       </c>
       <c r="F17" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G17" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H17" t="s">
         <v>95</v>
@@ -1818,13 +1845,13 @@
         <v>22</v>
       </c>
       <c r="K17" t="s">
-        <v>16</v>
+        <v>89</v>
       </c>
       <c r="L17" s="1">
-        <v>46264.125</v>
+        <v>46265.125</v>
       </c>
       <c r="M17" s="1">
-        <v>46262.64305005787</v>
+        <v>46265.60724832176</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
@@ -1832,60 +1859,60 @@
         <v>97</v>
       </c>
       <c r="B18" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C18" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D18" t="s">
         <v>98</v>
       </c>
       <c r="E18" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G18" t="s">
+        <v>30</v>
+      </c>
+      <c r="H18" t="s">
         <v>99</v>
       </c>
-      <c r="G18" t="s">
+      <c r="I18" t="s">
         <v>100</v>
       </c>
-      <c r="H18" t="s">
+      <c r="J18" t="s">
+        <v>33</v>
+      </c>
+      <c r="K18" t="s">
         <v>101</v>
       </c>
-      <c r="I18" t="s">
-        <v>102</v>
-      </c>
-      <c r="J18" t="s">
-        <v>19</v>
-      </c>
-      <c r="K18" t="s">
-        <v>103</v>
-      </c>
       <c r="L18" s="1">
-        <v>46263.125</v>
+        <v>46266.125</v>
       </c>
       <c r="M18" s="1">
-        <v>46261.88899761574</v>
+        <v>46264.545438518515</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B19" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" t="s">
+        <v>47</v>
+      </c>
+      <c r="D19" t="s">
+        <v>103</v>
+      </c>
+      <c r="E19" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" t="s">
         <v>104</v>
-      </c>
-      <c r="B19" t="s">
-        <v>42</v>
-      </c>
-      <c r="C19" t="s">
-        <v>15</v>
-      </c>
-      <c r="D19" t="s">
-        <v>70</v>
-      </c>
-      <c r="E19" t="s">
-        <v>17</v>
-      </c>
-      <c r="F19" t="s">
-        <v>71</v>
       </c>
       <c r="G19" t="s">
         <v>105</v>
@@ -1897,16 +1924,16 @@
         <v>107</v>
       </c>
       <c r="J19" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="K19" t="s">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="L19" s="1">
-        <v>46263.125</v>
+        <v>46264.125</v>
       </c>
       <c r="M19" s="1">
-        <v>46261.847652303244</v>
+        <v>46262.64305005787</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -1914,309 +1941,309 @@
         <v>108</v>
       </c>
       <c r="B20" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C20" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D20" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" t="s">
         <v>109</v>
       </c>
-      <c r="E20" t="s">
+      <c r="G20" t="s">
         <v>110</v>
       </c>
-      <c r="F20" t="s">
-        <v>26</v>
-      </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>111</v>
       </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>112</v>
       </c>
-      <c r="I20" t="s">
+      <c r="J20" t="s">
+        <v>33</v>
+      </c>
+      <c r="K20" t="s">
         <v>113</v>
-      </c>
-      <c r="J20" t="s">
-        <v>114</v>
-      </c>
-      <c r="K20" t="s">
-        <v>109</v>
       </c>
       <c r="L20" s="1">
         <v>46263.125</v>
       </c>
       <c r="M20" s="1">
-        <v>46261.76887157407</v>
+        <v>46261.88899761574</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>114</v>
+      </c>
+      <c r="B21" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" t="s">
+        <v>26</v>
+      </c>
+      <c r="D21" t="s">
+        <v>83</v>
+      </c>
+      <c r="E21" t="s">
+        <v>28</v>
+      </c>
+      <c r="F21" t="s">
+        <v>84</v>
+      </c>
+      <c r="G21" t="s">
         <v>115</v>
       </c>
-      <c r="B21" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21" t="s">
-        <v>15</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="H21" t="s">
         <v>116</v>
       </c>
-      <c r="E21" t="s">
-        <v>17</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="I21" t="s">
         <v>117</v>
       </c>
-      <c r="G21" t="s">
-        <v>72</v>
-      </c>
-      <c r="H21" t="s">
-        <v>118</v>
-      </c>
-      <c r="I21" t="s">
-        <v>119</v>
-      </c>
       <c r="J21" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="K21" t="s">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="L21" s="1">
         <v>46263.125</v>
       </c>
       <c r="M21" s="1">
-        <v>46261.75806057871</v>
+        <v>46261.847652303244</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>118</v>
+      </c>
+      <c r="B22" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" t="s">
+        <v>119</v>
+      </c>
+      <c r="E22" t="s">
         <v>120</v>
       </c>
-      <c r="B22" t="s">
-        <v>35</v>
-      </c>
-      <c r="C22" t="s">
-        <v>15</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="F22" t="s">
+        <v>42</v>
+      </c>
+      <c r="G22" t="s">
         <v>121</v>
       </c>
-      <c r="E22" t="s">
-        <v>110</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="H22" t="s">
         <v>122</v>
       </c>
-      <c r="G22" t="s">
+      <c r="I22" t="s">
         <v>123</v>
       </c>
-      <c r="H22" t="s">
+      <c r="J22" t="s">
         <v>124</v>
       </c>
-      <c r="I22" t="s">
-        <v>125</v>
-      </c>
-      <c r="J22" t="s">
-        <v>19</v>
-      </c>
       <c r="K22" t="s">
-        <v>19</v>
+        <v>119</v>
       </c>
       <c r="L22" s="1">
-        <v>46262.125</v>
+        <v>46263.125</v>
       </c>
       <c r="M22" s="1">
-        <v>46260.86106256944</v>
+        <v>46261.76887157407</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" t="s">
+        <v>56</v>
+      </c>
+      <c r="C23" t="s">
+        <v>26</v>
+      </c>
+      <c r="D23" t="s">
         <v>126</v>
       </c>
-      <c r="B23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C23" t="s">
-        <v>43</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
+        <v>28</v>
+      </c>
+      <c r="F23" t="s">
         <v>127</v>
       </c>
-      <c r="E23" t="s">
-        <v>25</v>
-      </c>
-      <c r="F23" t="s">
-        <v>38</v>
-      </c>
       <c r="G23" t="s">
+        <v>85</v>
+      </c>
+      <c r="H23" t="s">
         <v>128</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>129</v>
       </c>
-      <c r="I23" t="s">
-        <v>130</v>
-      </c>
       <c r="J23" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="K23" t="s">
-        <v>131</v>
+        <v>72</v>
       </c>
       <c r="L23" s="1">
-        <v>46262.125</v>
+        <v>46263.125</v>
       </c>
       <c r="M23" s="1">
-        <v>46260.789700995374</v>
+        <v>46261.75806057871</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>130</v>
+      </c>
+      <c r="B24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C24" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" t="s">
+        <v>131</v>
+      </c>
+      <c r="E24" t="s">
+        <v>120</v>
+      </c>
+      <c r="F24" t="s">
         <v>132</v>
       </c>
-      <c r="B24" t="s">
-        <v>42</v>
-      </c>
-      <c r="C24" t="s">
-        <v>15</v>
-      </c>
-      <c r="D24" t="s">
-        <v>70</v>
-      </c>
-      <c r="E24" t="s">
-        <v>17</v>
-      </c>
-      <c r="F24" t="s">
-        <v>71</v>
-      </c>
       <c r="G24" t="s">
-        <v>72</v>
+        <v>133</v>
       </c>
       <c r="H24" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I24" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J24" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="K24" t="s">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="L24" s="1">
         <v>46262.125</v>
       </c>
       <c r="M24" s="1">
-        <v>46260.77278251157</v>
+        <v>46260.86106256944</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B25" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C25" t="s">
         <v>15</v>
       </c>
       <c r="D25" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E25" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F25" t="s">
-        <v>77</v>
+        <v>52</v>
       </c>
       <c r="G25" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H25" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I25" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J25" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="K25" t="s">
-        <v>76</v>
+        <v>23</v>
       </c>
       <c r="L25" s="1">
         <v>46262.125</v>
       </c>
       <c r="M25" s="1">
-        <v>46260.751369895836</v>
+        <v>46260.789700995374</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B26" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C26" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="D26" t="s">
-        <v>141</v>
+        <v>83</v>
       </c>
       <c r="E26" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F26" t="s">
+        <v>84</v>
+      </c>
+      <c r="G26" t="s">
+        <v>85</v>
+      </c>
+      <c r="H26" t="s">
         <v>142</v>
       </c>
-      <c r="G26" t="s">
-        <v>100</v>
-      </c>
-      <c r="H26" t="s">
+      <c r="I26" t="s">
         <v>143</v>
       </c>
-      <c r="I26" t="s">
-        <v>144</v>
-      </c>
       <c r="J26" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="K26" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="L26" s="1">
-        <v>46260.125</v>
+        <v>46262.125</v>
       </c>
       <c r="M26" s="1">
-        <v>46260.68583916667</v>
+        <v>46260.77278251157</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>144</v>
+      </c>
+      <c r="B27" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" t="s">
+        <v>26</v>
+      </c>
+      <c r="D27" t="s">
         <v>145</v>
-      </c>
-      <c r="B27" t="s">
-        <v>42</v>
-      </c>
-      <c r="C27" t="s">
-        <v>15</v>
-      </c>
-      <c r="D27" t="s">
-        <v>146</v>
       </c>
       <c r="E27" t="s">
         <v>17</v>
       </c>
       <c r="F27" t="s">
-        <v>18</v>
+        <v>90</v>
       </c>
       <c r="G27" t="s">
-        <v>100</v>
+        <v>146</v>
       </c>
       <c r="H27" t="s">
         <v>147</v>
@@ -2228,13 +2255,13 @@
         <v>22</v>
       </c>
       <c r="K27" t="s">
-        <v>16</v>
+        <v>89</v>
       </c>
       <c r="L27" s="1">
         <v>46262.125</v>
       </c>
       <c r="M27" s="1">
-        <v>46260.610648877315</v>
+        <v>46260.751369895836</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
@@ -2242,22 +2269,22 @@
         <v>149</v>
       </c>
       <c r="B28" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C28" t="s">
         <v>15</v>
       </c>
       <c r="D28" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="E28" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F28" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G28" t="s">
-        <v>151</v>
+        <v>110</v>
       </c>
       <c r="H28" t="s">
         <v>152</v>
@@ -2266,39 +2293,39 @@
         <v>153</v>
       </c>
       <c r="J28" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="K28" t="s">
-        <v>154</v>
+        <v>59</v>
       </c>
       <c r="L28" s="1">
-        <v>46262.125</v>
+        <v>46260.125</v>
       </c>
       <c r="M28" s="1">
-        <v>46260.562727013894</v>
+        <v>46260.68583916667</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>154</v>
+      </c>
+      <c r="B29" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29" t="s">
         <v>155</v>
       </c>
-      <c r="B29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C29" t="s">
-        <v>15</v>
-      </c>
-      <c r="D29" t="s">
-        <v>141</v>
-      </c>
       <c r="E29" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F29" t="s">
-        <v>142</v>
+        <v>36</v>
       </c>
       <c r="G29" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="H29" t="s">
         <v>156</v>
@@ -2307,16 +2334,16 @@
         <v>157</v>
       </c>
       <c r="J29" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="K29" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="L29" s="1">
-        <v>46260.125</v>
+        <v>46262.125</v>
       </c>
       <c r="M29" s="1">
-        <v>46260.553795775464</v>
+        <v>46260.610648877315</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
@@ -2324,63 +2351,63 @@
         <v>158</v>
       </c>
       <c r="B30" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C30" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D30" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E30" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F30" t="s">
-        <v>142</v>
+        <v>159</v>
       </c>
       <c r="G30" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H30" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I30" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J30" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="K30" t="s">
-        <v>46</v>
+        <v>163</v>
       </c>
       <c r="L30" s="1">
-        <v>46261.125</v>
+        <v>46262.125</v>
       </c>
       <c r="M30" s="1">
-        <v>46259.760144201384</v>
+        <v>46260.562727013894</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B31" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C31" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D31" t="s">
-        <v>163</v>
+        <v>150</v>
       </c>
       <c r="E31" t="s">
         <v>17</v>
       </c>
       <c r="F31" t="s">
-        <v>86</v>
+        <v>151</v>
       </c>
       <c r="G31" t="s">
-        <v>164</v>
+        <v>110</v>
       </c>
       <c r="H31" t="s">
         <v>165</v>
@@ -2389,98 +2416,98 @@
         <v>166</v>
       </c>
       <c r="J31" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="K31" t="s">
-        <v>167</v>
+        <v>59</v>
       </c>
       <c r="L31" s="1">
         <v>46260.125</v>
       </c>
       <c r="M31" s="1">
-        <v>46258.85121311343</v>
+        <v>46260.553795775464</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B32" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C32" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D32" t="s">
-        <v>169</v>
+        <v>150</v>
       </c>
       <c r="E32" t="s">
         <v>17</v>
       </c>
       <c r="F32" t="s">
+        <v>151</v>
+      </c>
+      <c r="G32" t="s">
+        <v>168</v>
+      </c>
+      <c r="H32" t="s">
+        <v>169</v>
+      </c>
+      <c r="I32" t="s">
         <v>170</v>
-      </c>
-      <c r="G32" t="s">
-        <v>171</v>
-      </c>
-      <c r="H32" t="s">
-        <v>172</v>
-      </c>
-      <c r="I32" t="s">
-        <v>173</v>
       </c>
       <c r="J32" t="s">
         <v>22</v>
       </c>
       <c r="K32" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="L32" s="1">
-        <v>46257.125</v>
+        <v>46261.125</v>
       </c>
       <c r="M32" s="1">
-        <v>46255.90268423611</v>
+        <v>46259.760144201384</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>171</v>
+      </c>
+      <c r="B33" t="s">
+        <v>56</v>
+      </c>
+      <c r="C33" t="s">
+        <v>47</v>
+      </c>
+      <c r="D33" t="s">
+        <v>172</v>
+      </c>
+      <c r="E33" t="s">
+        <v>28</v>
+      </c>
+      <c r="F33" t="s">
+        <v>29</v>
+      </c>
+      <c r="G33" t="s">
+        <v>173</v>
+      </c>
+      <c r="H33" t="s">
         <v>174</v>
       </c>
-      <c r="B33" t="s">
-        <v>42</v>
-      </c>
-      <c r="C33" t="s">
-        <v>15</v>
-      </c>
-      <c r="D33" t="s">
-        <v>37</v>
-      </c>
-      <c r="E33" t="s">
-        <v>25</v>
-      </c>
-      <c r="F33" t="s">
-        <v>38</v>
-      </c>
-      <c r="G33" t="s">
-        <v>19</v>
-      </c>
-      <c r="H33" t="s">
+      <c r="I33" t="s">
         <v>175</v>
       </c>
-      <c r="I33" t="s">
+      <c r="J33" t="s">
+        <v>33</v>
+      </c>
+      <c r="K33" t="s">
         <v>176</v>
       </c>
-      <c r="J33" t="s">
-        <v>29</v>
-      </c>
-      <c r="K33" t="s">
-        <v>131</v>
-      </c>
       <c r="L33" s="1">
-        <v>46257.125</v>
+        <v>46260.125</v>
       </c>
       <c r="M33" s="1">
-        <v>46255.846485312504</v>
+        <v>46258.85121311343</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
@@ -2488,142 +2515,142 @@
         <v>177</v>
       </c>
       <c r="B34" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C34" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D34" t="s">
         <v>178</v>
       </c>
       <c r="E34" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F34" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="G34" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H34" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="I34" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J34" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="K34" t="s">
-        <v>154</v>
+        <v>81</v>
       </c>
       <c r="L34" s="1">
         <v>46257.125</v>
       </c>
       <c r="M34" s="1">
-        <v>46255.741482881946</v>
+        <v>46255.90268423611</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B35" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C35" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="D35" t="s">
-        <v>183</v>
+        <v>16</v>
       </c>
       <c r="E35" t="s">
         <v>17</v>
       </c>
       <c r="F35" t="s">
+        <v>52</v>
+      </c>
+      <c r="G35" t="s">
+        <v>33</v>
+      </c>
+      <c r="H35" t="s">
         <v>184</v>
       </c>
-      <c r="G35" t="s">
+      <c r="I35" t="s">
         <v>185</v>
-      </c>
-      <c r="H35" t="s">
-        <v>186</v>
-      </c>
-      <c r="I35" t="s">
-        <v>187</v>
       </c>
       <c r="J35" t="s">
         <v>22</v>
       </c>
       <c r="K35" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="L35" s="1">
         <v>46257.125</v>
       </c>
       <c r="M35" s="1">
-        <v>46255.72513931713</v>
+        <v>46255.846485312504</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B36" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C36" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D36" t="s">
-        <v>163</v>
+        <v>187</v>
       </c>
       <c r="E36" t="s">
         <v>17</v>
       </c>
       <c r="F36" t="s">
-        <v>86</v>
+        <v>159</v>
       </c>
       <c r="G36" t="s">
+        <v>188</v>
+      </c>
+      <c r="H36" t="s">
         <v>189</v>
       </c>
-      <c r="H36" t="s">
+      <c r="I36" t="s">
         <v>190</v>
       </c>
-      <c r="I36" t="s">
-        <v>191</v>
-      </c>
       <c r="J36" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="K36" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="L36" s="1">
         <v>46257.125</v>
       </c>
       <c r="M36" s="1">
-        <v>46255.69151269676</v>
+        <v>46255.741482881946</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>191</v>
+      </c>
+      <c r="B37" t="s">
+        <v>56</v>
+      </c>
+      <c r="C37" t="s">
+        <v>15</v>
+      </c>
+      <c r="D37" t="s">
         <v>192</v>
       </c>
-      <c r="B37" t="s">
-        <v>42</v>
-      </c>
-      <c r="C37" t="s">
-        <v>32</v>
-      </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
+        <v>28</v>
+      </c>
+      <c r="F37" t="s">
         <v>193</v>
-      </c>
-      <c r="E37" t="s">
-        <v>17</v>
-      </c>
-      <c r="F37" t="s">
-        <v>86</v>
       </c>
       <c r="G37" t="s">
         <v>194</v>
@@ -2635,16 +2662,16 @@
         <v>196</v>
       </c>
       <c r="J37" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="K37" t="s">
-        <v>167</v>
+        <v>35</v>
       </c>
       <c r="L37" s="1">
         <v>46257.125</v>
       </c>
       <c r="M37" s="1">
-        <v>46255.6164808912</v>
+        <v>46255.72513931713</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
@@ -2652,183 +2679,183 @@
         <v>197</v>
       </c>
       <c r="B38" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C38" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D38" t="s">
-        <v>24</v>
+        <v>172</v>
       </c>
       <c r="E38" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F38" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G38" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="H38" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I38" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J38" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="K38" t="s">
-        <v>30</v>
+        <v>176</v>
       </c>
       <c r="L38" s="1">
         <v>46257.125</v>
       </c>
       <c r="M38" s="1">
-        <v>46255.58180528935</v>
+        <v>46255.69151269676</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B39" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C39" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="D39" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E39" t="s">
-        <v>110</v>
+        <v>28</v>
       </c>
       <c r="F39" t="s">
-        <v>202</v>
+        <v>29</v>
       </c>
       <c r="G39" t="s">
-        <v>100</v>
+        <v>203</v>
       </c>
       <c r="H39" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I39" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="J39" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="K39" t="s">
-        <v>121</v>
+        <v>176</v>
       </c>
       <c r="L39" s="1">
-        <v>46255.125</v>
+        <v>46257.125</v>
       </c>
       <c r="M39" s="1">
-        <v>46255.57480164352</v>
+        <v>46255.6164808912</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B40" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C40" t="s">
         <v>15</v>
       </c>
       <c r="D40" t="s">
-        <v>206</v>
+        <v>41</v>
       </c>
       <c r="E40" t="s">
-        <v>110</v>
+        <v>17</v>
       </c>
       <c r="F40" t="s">
+        <v>42</v>
+      </c>
+      <c r="G40" t="s">
+        <v>42</v>
+      </c>
+      <c r="H40" t="s">
         <v>207</v>
       </c>
-      <c r="G40" t="s">
+      <c r="I40" t="s">
         <v>208</v>
       </c>
-      <c r="H40" t="s">
-        <v>209</v>
-      </c>
-      <c r="I40" t="s">
-        <v>210</v>
-      </c>
       <c r="J40" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="K40" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="L40" s="1">
         <v>46257.125</v>
       </c>
       <c r="M40" s="1">
-        <v>46255.450155185186</v>
+        <v>46255.58180528935</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>209</v>
+      </c>
+      <c r="B41" t="s">
+        <v>56</v>
+      </c>
+      <c r="C41" t="s">
+        <v>26</v>
+      </c>
+      <c r="D41" t="s">
+        <v>210</v>
+      </c>
+      <c r="E41" t="s">
+        <v>120</v>
+      </c>
+      <c r="F41" t="s">
         <v>211</v>
       </c>
-      <c r="B41" t="s">
-        <v>42</v>
-      </c>
-      <c r="C41" t="s">
-        <v>32</v>
-      </c>
-      <c r="D41" t="s">
+      <c r="G41" t="s">
+        <v>110</v>
+      </c>
+      <c r="H41" t="s">
         <v>212</v>
       </c>
-      <c r="E41" t="s">
-        <v>110</v>
-      </c>
-      <c r="F41" t="s">
+      <c r="I41" t="s">
         <v>213</v>
       </c>
-      <c r="G41" t="s">
-        <v>72</v>
-      </c>
-      <c r="H41" t="s">
-        <v>214</v>
-      </c>
-      <c r="I41" t="s">
-        <v>215</v>
-      </c>
       <c r="J41" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="K41" t="s">
-        <v>212</v>
+        <v>131</v>
       </c>
       <c r="L41" s="1">
-        <v>46257.125</v>
+        <v>46255.125</v>
       </c>
       <c r="M41" s="1">
-        <v>46255.44403424769</v>
+        <v>46255.57480164352</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>214</v>
+      </c>
+      <c r="B42" t="s">
+        <v>56</v>
+      </c>
+      <c r="C42" t="s">
+        <v>26</v>
+      </c>
+      <c r="D42" t="s">
+        <v>215</v>
+      </c>
+      <c r="E42" t="s">
+        <v>120</v>
+      </c>
+      <c r="F42" t="s">
         <v>216</v>
-      </c>
-      <c r="B42" t="s">
-        <v>42</v>
-      </c>
-      <c r="C42" t="s">
-        <v>43</v>
-      </c>
-      <c r="D42" t="s">
-        <v>98</v>
-      </c>
-      <c r="E42" t="s">
-        <v>17</v>
-      </c>
-      <c r="F42" t="s">
-        <v>99</v>
       </c>
       <c r="G42" t="s">
         <v>217</v>
@@ -2843,13 +2870,13 @@
         <v>22</v>
       </c>
       <c r="K42" t="s">
-        <v>103</v>
+        <v>45</v>
       </c>
       <c r="L42" s="1">
-        <v>46256.125</v>
+        <v>46257.125</v>
       </c>
       <c r="M42" s="1">
-        <v>46254.83730204861</v>
+        <v>46255.450155185186</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
@@ -2857,101 +2884,101 @@
         <v>220</v>
       </c>
       <c r="B43" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C43" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="D43" t="s">
-        <v>163</v>
+        <v>221</v>
       </c>
       <c r="E43" t="s">
-        <v>17</v>
+        <v>120</v>
       </c>
       <c r="F43" t="s">
-        <v>86</v>
+        <v>222</v>
       </c>
       <c r="G43" t="s">
+        <v>85</v>
+      </c>
+      <c r="H43" t="s">
+        <v>223</v>
+      </c>
+      <c r="I43" t="s">
+        <v>224</v>
+      </c>
+      <c r="J43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K43" t="s">
         <v>221</v>
       </c>
-      <c r="H43" t="s">
-        <v>222</v>
-      </c>
-      <c r="I43" t="s">
-        <v>223</v>
-      </c>
-      <c r="J43" t="s">
-        <v>22</v>
-      </c>
-      <c r="K43" t="s">
-        <v>103</v>
-      </c>
       <c r="L43" s="1">
-        <v>46256.125</v>
+        <v>46257.125</v>
       </c>
       <c r="M43" s="1">
-        <v>46254.637882800926</v>
+        <v>46255.44403424769</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B44" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C44" t="s">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="D44" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="E44" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F44" t="s">
-        <v>71</v>
+        <v>109</v>
       </c>
       <c r="G44" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H44" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="I44" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="J44" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="K44" t="s">
-        <v>68</v>
+        <v>113</v>
       </c>
       <c r="L44" s="1">
-        <v>46255.125</v>
+        <v>46256.125</v>
       </c>
       <c r="M44" s="1">
-        <v>46253.62513393519</v>
+        <v>46254.83730204861</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B45" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C45" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="D45" t="s">
-        <v>229</v>
+        <v>172</v>
       </c>
       <c r="E45" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F45" t="s">
-        <v>150</v>
+        <v>29</v>
       </c>
       <c r="G45" t="s">
         <v>230</v>
@@ -2963,16 +2990,16 @@
         <v>232</v>
       </c>
       <c r="J45" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="K45" t="s">
-        <v>154</v>
+        <v>113</v>
       </c>
       <c r="L45" s="1">
-        <v>46255.125</v>
+        <v>46256.125</v>
       </c>
       <c r="M45" s="1">
-        <v>46253.58023178241</v>
+        <v>46254.637882800926</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
@@ -2980,39 +3007,121 @@
         <v>233</v>
       </c>
       <c r="B46" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="C46" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="D46" t="s">
-        <v>206</v>
+        <v>83</v>
       </c>
       <c r="E46" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F46" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G46" t="s">
-        <v>137</v>
+        <v>234</v>
       </c>
       <c r="H46" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="I46" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="J46" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="K46" t="s">
-        <v>19</v>
+        <v>81</v>
       </c>
       <c r="L46" s="1">
         <v>46255.125</v>
       </c>
       <c r="M46" s="1">
+        <v>46253.62513393519</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>237</v>
+      </c>
+      <c r="B47" t="s">
+        <v>56</v>
+      </c>
+      <c r="C47" t="s">
+        <v>26</v>
+      </c>
+      <c r="D47" t="s">
+        <v>238</v>
+      </c>
+      <c r="E47" t="s">
+        <v>17</v>
+      </c>
+      <c r="F47" t="s">
+        <v>159</v>
+      </c>
+      <c r="G47" t="s">
+        <v>239</v>
+      </c>
+      <c r="H47" t="s">
+        <v>240</v>
+      </c>
+      <c r="I47" t="s">
+        <v>241</v>
+      </c>
+      <c r="J47" t="s">
+        <v>33</v>
+      </c>
+      <c r="K47" t="s">
+        <v>163</v>
+      </c>
+      <c r="L47" s="1">
+        <v>46255.125</v>
+      </c>
+      <c r="M47" s="1">
+        <v>46253.58023178241</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>242</v>
+      </c>
+      <c r="B48" t="s">
+        <v>50</v>
+      </c>
+      <c r="C48" t="s">
+        <v>47</v>
+      </c>
+      <c r="D48" t="s">
+        <v>215</v>
+      </c>
+      <c r="E48" t="s">
+        <v>17</v>
+      </c>
+      <c r="F48" t="s">
+        <v>90</v>
+      </c>
+      <c r="G48" t="s">
+        <v>146</v>
+      </c>
+      <c r="H48" t="s">
+        <v>243</v>
+      </c>
+      <c r="I48" t="s">
+        <v>244</v>
+      </c>
+      <c r="J48" t="s">
+        <v>33</v>
+      </c>
+      <c r="K48" t="s">
+        <v>33</v>
+      </c>
+      <c r="L48" s="1">
+        <v>46255.125</v>
+      </c>
+      <c r="M48" s="1">
         <v>46253.549469791666</v>
       </c>
     </row>

</xml_diff>